<commit_message>
Update MLB hitter fantasy scores 2026-07-23 (2026-07-22 08:40 PM)
</commit_message>
<xml_diff>
--- a/PRIZEPICKS_HITTER_AI_V6_TOP30_2026_07_23.xlsx
+++ b/PRIZEPICKS_HITTER_AI_V6_TOP30_2026_07_23.xlsx
@@ -2915,7 +2915,7 @@
       </c>
       <c r="HO2" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP2" s="3" t="n">
@@ -3824,7 +3824,7 @@
       </c>
       <c r="HO3" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP3" s="3" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="HO4" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP4" s="3" t="n">
@@ -5634,7 +5634,7 @@
       </c>
       <c r="HO5" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP5" s="3" t="n">
@@ -6543,7 +6543,7 @@
       </c>
       <c r="HO6" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP6" s="3" t="n">
@@ -7452,7 +7452,7 @@
       </c>
       <c r="HO7" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP7" s="3" t="n">
@@ -8353,7 +8353,7 @@
       </c>
       <c r="HO8" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP8" s="3" t="n">
@@ -9262,7 +9262,7 @@
       </c>
       <c r="HO9" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP9" s="3" t="n">
@@ -10171,7 +10171,7 @@
       </c>
       <c r="HO10" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP10" s="3" t="n">
@@ -11080,7 +11080,7 @@
       </c>
       <c r="HO11" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP11" s="3" t="n">
@@ -11989,7 +11989,7 @@
       </c>
       <c r="HO12" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP12" s="3" t="n">
@@ -12898,7 +12898,7 @@
       </c>
       <c r="HO13" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP13" s="3" t="n">
@@ -13807,7 +13807,7 @@
       </c>
       <c r="HO14" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP14" s="3" t="n">
@@ -14716,7 +14716,7 @@
       </c>
       <c r="HO15" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP15" s="3" t="n">
@@ -15617,7 +15617,7 @@
       </c>
       <c r="HO16" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP16" s="3" t="n">
@@ -16526,7 +16526,7 @@
       </c>
       <c r="HO17" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP17" s="3" t="n">
@@ -17427,7 +17427,7 @@
       </c>
       <c r="HO18" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP18" s="3" t="n">
@@ -18336,7 +18336,7 @@
       </c>
       <c r="HO19" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP19" s="3" t="n">
@@ -19237,7 +19237,7 @@
       </c>
       <c r="HO20" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP20" s="3" t="n">
@@ -20146,7 +20146,7 @@
       </c>
       <c r="HO21" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP21" s="3" t="n">
@@ -21055,7 +21055,7 @@
       </c>
       <c r="HO22" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP22" s="3" t="n">
@@ -21964,7 +21964,7 @@
       </c>
       <c r="HO23" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP23" s="3" t="n">
@@ -22873,7 +22873,7 @@
       </c>
       <c r="HO24" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP24" s="3" t="n">
@@ -23782,7 +23782,7 @@
       </c>
       <c r="HO25" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP25" s="3" t="n">
@@ -24691,7 +24691,7 @@
       </c>
       <c r="HO26" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP26" s="3" t="n">
@@ -25600,7 +25600,7 @@
       </c>
       <c r="HO27" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP27" s="3" t="n">
@@ -26509,7 +26509,7 @@
       </c>
       <c r="HO28" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP28" s="3" t="n">
@@ -27418,7 +27418,7 @@
       </c>
       <c r="HO29" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP29" s="3" t="n">
@@ -28327,7 +28327,7 @@
       </c>
       <c r="HO30" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP30" s="3" t="n">
@@ -29236,7 +29236,7 @@
       </c>
       <c r="HO31" s="4" t="inlineStr">
         <is>
-          <t>Raw (calibration off)</t>
+          <t>Raw</t>
         </is>
       </c>
       <c r="HP31" s="3" t="n">

</xml_diff>